<commit_message>
marked the same cells
</commit_message>
<xml_diff>
--- a/Cortana/cell_list_investigation/zombies_all_anova_passed_cells--used for grant.xlsx
+++ b/Cortana/cell_list_investigation/zombies_all_anova_passed_cells--used for grant.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="95">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t xml:space="preserve">(200.0, 700.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same unit</t>
   </si>
   <si>
     <t xml:space="preserve">(250.0, 600.0)</t>
@@ -569,13 +572,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1023" style="0" width="9.14"/>
   </cols>
   <sheetData>
@@ -1513,6 +1516,9 @@
       <c r="E55" s="12" t="n">
         <v>0.00665026125701438</v>
       </c>
+      <c r="F55" s="12" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="56" s="12" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="n">
@@ -1530,6 +1536,9 @@
       <c r="E56" s="12" t="n">
         <v>0.006289624603342</v>
       </c>
+      <c r="F56" s="12" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="57" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="n">
@@ -1547,6 +1556,9 @@
       <c r="E57" s="10" t="n">
         <v>0.00763427299537475</v>
       </c>
+      <c r="F57" s="10" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="58" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="n">
@@ -1564,6 +1576,9 @@
       <c r="E58" s="10" t="n">
         <v>0.006514719781525</v>
       </c>
+      <c r="F58" s="10" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="n">
@@ -1573,10 +1588,10 @@
         <v>1</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E59" s="0" t="n">
         <v>0.004480491399968</v>
@@ -1590,7 +1605,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>10</v>
@@ -1624,7 +1639,7 @@
         <v>1</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D62" s="0" t="s">
         <v>57</v>
@@ -1658,10 +1673,10 @@
         <v>1</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>0.0156939900887875</v>
@@ -1678,7 +1693,7 @@
         <v>34</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>0.0307663890018702</v>
@@ -1695,7 +1710,7 @@
         <v>9</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0.0363170926256485</v>
@@ -1709,7 +1724,7 @@
         <v>3</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D67" s="0" t="s">
         <v>59</v>
@@ -1726,10 +1741,10 @@
         <v>4</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E68" s="0" t="n">
         <v>0.0341434537209639</v>
@@ -1743,10 +1758,10 @@
         <v>4</v>
       </c>
       <c r="C69" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D69" s="0" t="s">
         <v>83</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>82</v>
       </c>
       <c r="E69" s="0" t="n">
         <v>0.0420897306933529</v>
@@ -1760,10 +1775,10 @@
         <v>1</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E70" s="0" t="n">
         <v>0.0387635591675108</v>
@@ -1777,10 +1792,10 @@
         <v>1</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E71" s="0" t="n">
         <v>2.86335363152876E-005</v>
@@ -1811,10 +1826,10 @@
         <v>4</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E73" s="0" t="n">
         <v>0.0423018416670973</v>
@@ -1828,10 +1843,10 @@
         <v>2</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E74" s="0" t="n">
         <v>0.0379316883083251</v>
@@ -1845,10 +1860,10 @@
         <v>3</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E75" s="0" t="n">
         <v>0.0374272936245397</v>
@@ -1865,7 +1880,7 @@
         <v>30</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E76" s="0" t="n">
         <v>0.0108022991106536</v>
@@ -1873,8 +1888,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
began sorting the grant unsorted cells and been recording them on zombies_all_anova_passed_cells--used for grant.xlsx file
</commit_message>
<xml_diff>
--- a/Cortana/cell_list_investigation/zombies_all_anova_passed_cells--used for grant.xlsx
+++ b/Cortana/cell_list_investigation/zombies_all_anova_passed_cells--used for grant.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="100">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -37,6 +37,12 @@
     <t xml:space="preserve">P Value</t>
   </si>
   <si>
+    <t xml:space="preserve">Sorted?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Units</t>
+  </si>
+  <si>
     <t xml:space="preserve">(0.0, 300.0)</t>
   </si>
   <si>
@@ -55,6 +61,9 @@
     <t xml:space="preserve">Channel.C_020</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">(0.0, 2000.0)</t>
   </si>
   <si>
@@ -100,6 +109,9 @@
     <t xml:space="preserve">Channel.C_006</t>
   </si>
   <si>
+    <t xml:space="preserve">Unit 2 appeared late in the experiment</t>
+  </si>
+  <si>
     <t xml:space="preserve">(200.0, 650.0)</t>
   </si>
   <si>
@@ -176,6 +188,9 @@
   </si>
   <si>
     <t xml:space="preserve">Channel.C_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">should be removed (sorted already)</t>
   </si>
   <si>
     <t xml:space="preserve">(500.0, 850.0)</t>
@@ -572,13 +587,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1023" style="0" width="9.14"/>
   </cols>
   <sheetData>
@@ -598,6 +614,12 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
@@ -607,10 +629,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E2" s="0" t="n">
         <v>0.030965715390678</v>
@@ -624,10 +646,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0.0224122204061938</v>
@@ -641,13 +663,19 @@
         <v>2</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>0.00488467703525351</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -658,10 +686,10 @@
         <v>3</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E5" s="0" t="n">
         <v>0.0001048561426</v>
@@ -675,10 +703,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E6" s="0" t="n">
         <v>0.031938468862498</v>
@@ -692,10 +720,10 @@
         <v>3</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E7" s="0" t="n">
         <v>0.0459134288678394</v>
@@ -709,10 +737,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" s="0" t="n">
         <v>0.000205299212230494</v>
@@ -726,10 +754,10 @@
         <v>3</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E9" s="0" t="n">
         <v>0.000219903122149023</v>
@@ -743,10 +771,10 @@
         <v>3</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E10" s="0" t="n">
         <v>0.03527854547184</v>
@@ -760,10 +788,10 @@
         <v>3</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E11" s="0" t="n">
         <v>0.00127725376352979</v>
@@ -777,13 +805,22 @@
         <v>4</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E12" s="0" t="n">
         <v>0.00707558272740489</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="0" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="13" s="6" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -794,10 +831,10 @@
         <v>4</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>0.00159172655600108</v>
@@ -811,10 +848,10 @@
         <v>4</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>0.000378311542831</v>
@@ -828,13 +865,19 @@
         <v>4</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>0.0470807977888419</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" s="6" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -845,10 +888,10 @@
         <v>1</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>7.5061489843254E-007</v>
@@ -862,10 +905,10 @@
         <v>1</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>1.05830081034659E-006</v>
@@ -879,10 +922,10 @@
         <v>1</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E18" s="8" t="n">
         <v>5.0489588623909E-005</v>
@@ -896,10 +939,10 @@
         <v>1</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>2.13976612550698E-005</v>
@@ -913,10 +956,10 @@
         <v>2</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>1.51626385288723E-011</v>
@@ -930,10 +973,10 @@
         <v>2</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E21" s="10" t="n">
         <v>7.55699317281293E-011</v>
@@ -947,10 +990,10 @@
         <v>2</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E22" s="0" t="n">
         <v>1.66280772505988E-005</v>
@@ -964,10 +1007,10 @@
         <v>3</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E23" s="10" t="n">
         <v>4.82855775313535E-005</v>
@@ -981,10 +1024,10 @@
         <v>3</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E24" s="10" t="n">
         <v>2.33114874428906E-005</v>
@@ -998,10 +1041,10 @@
         <v>3</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E25" s="12" t="n">
         <v>0.0353088450142687</v>
@@ -1015,10 +1058,10 @@
         <v>3</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E26" s="12" t="n">
         <v>0.012545428798116</v>
@@ -1032,10 +1075,10 @@
         <v>3</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E27" s="10" t="n">
         <v>0.00104884300249579</v>
@@ -1049,10 +1092,10 @@
         <v>3</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E28" s="10" t="n">
         <v>0.038781460115805</v>
@@ -1066,10 +1109,10 @@
         <v>3</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E29" s="12" t="n">
         <v>0.0395639912055182</v>
@@ -1083,10 +1126,10 @@
         <v>3</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E30" s="12" t="n">
         <v>0.042377881281726</v>
@@ -1100,10 +1143,10 @@
         <v>4</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E31" s="0" t="n">
         <v>0.0410304872185249</v>
@@ -1117,10 +1160,10 @@
         <v>4</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E32" s="10" t="n">
         <v>0.00168825852991398</v>
@@ -1134,10 +1177,10 @@
         <v>4</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E33" s="10" t="n">
         <v>0.011944886356068</v>
@@ -1151,10 +1194,10 @@
         <v>4</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E34" s="14" t="n">
         <v>0.00016076355362287</v>
@@ -1168,10 +1211,10 @@
         <v>4</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E35" s="14" t="n">
         <v>0.00029232953002</v>
@@ -1185,13 +1228,16 @@
         <v>1</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E36" s="16" t="n">
         <v>0.00986766757997</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="37" s="16" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1202,10 +1248,10 @@
         <v>1</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E37" s="16" t="n">
         <v>0.0451555088063392</v>
@@ -1219,10 +1265,10 @@
         <v>2</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E38" s="0" t="n">
         <v>0.000937658799145095</v>
@@ -1236,10 +1282,10 @@
         <v>2</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E39" s="0" t="n">
         <v>0.0146381959778083</v>
@@ -1253,10 +1299,10 @@
         <v>2</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E40" s="0" t="n">
         <v>0.0416051516577862</v>
@@ -1270,13 +1316,19 @@
         <v>3</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E41" s="0" t="n">
         <v>0.0179426294938499</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1287,13 +1339,19 @@
         <v>2</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E42" s="0" t="n">
         <v>0.0299065586144327</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1304,13 +1362,19 @@
         <v>2</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E43" s="0" t="n">
         <v>0.0207972809620275</v>
+      </c>
+      <c r="F43" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1321,13 +1385,19 @@
         <v>2</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E44" s="0" t="n">
         <v>0.0109178027087272</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1338,13 +1408,19 @@
         <v>2</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E45" s="0" t="n">
         <v>0.0421362181422794</v>
+      </c>
+      <c r="F45" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="46" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1355,13 +1431,19 @@
         <v>1</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E46" s="10" t="n">
         <v>3.38332280973613E-005</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" s="10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1372,13 +1454,19 @@
         <v>1</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E47" s="10" t="n">
         <v>1.49682454822413E-005</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1389,13 +1477,19 @@
         <v>1</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="E48" s="0" t="n">
         <v>0.0416891737433396</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G48" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1406,10 +1500,10 @@
         <v>3</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E49" s="0" t="n">
         <v>0.009555414268796</v>
@@ -1423,10 +1517,10 @@
         <v>3</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E50" s="10" t="n">
         <v>0.00580553000234327</v>
@@ -1440,10 +1534,10 @@
         <v>3</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E51" s="10" t="n">
         <v>0.001540377255957</v>
@@ -1457,10 +1551,10 @@
         <v>2</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E52" s="0" t="n">
         <v>0.01126620279013</v>
@@ -1474,10 +1568,10 @@
         <v>3</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E53" s="0" t="n">
         <v>0.0163236212793226</v>
@@ -1491,10 +1585,10 @@
         <v>3</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E54" s="0" t="n">
         <v>0.0494787080515314</v>
@@ -1508,16 +1602,16 @@
         <v>4</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E55" s="12" t="n">
         <v>0.00665026125701438</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="56" s="12" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1528,16 +1622,16 @@
         <v>4</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E56" s="12" t="n">
         <v>0.006289624603342</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="57" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1548,16 +1642,16 @@
         <v>4</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E57" s="10" t="n">
         <v>0.00763427299537475</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="58" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,16 +1662,16 @@
         <v>4</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E58" s="10" t="n">
         <v>0.006514719781525</v>
       </c>
       <c r="F58" s="10" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1588,10 +1682,10 @@
         <v>1</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E59" s="0" t="n">
         <v>0.004480491399968</v>
@@ -1605,10 +1699,10 @@
         <v>1</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0.011429781534636</v>
@@ -1622,10 +1716,10 @@
         <v>1</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>0.000335148307695</v>
@@ -1639,10 +1733,10 @@
         <v>1</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>0.0332634341315389</v>
@@ -1656,10 +1750,10 @@
         <v>2</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E63" s="0" t="n">
         <v>0.00479018499791497</v>
@@ -1673,10 +1767,10 @@
         <v>1</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>0.0156939900887875</v>
@@ -1690,10 +1784,10 @@
         <v>1</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>0.0307663890018702</v>
@@ -1707,10 +1801,10 @@
         <v>3</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0.0363170926256485</v>
@@ -1724,10 +1818,10 @@
         <v>3</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>0.0185877355832485</v>
@@ -1741,10 +1835,10 @@
         <v>4</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E68" s="0" t="n">
         <v>0.0341434537209639</v>
@@ -1758,10 +1852,10 @@
         <v>4</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E69" s="0" t="n">
         <v>0.0420897306933529</v>
@@ -1775,10 +1869,10 @@
         <v>1</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E70" s="0" t="n">
         <v>0.0387635591675108</v>
@@ -1792,10 +1886,10 @@
         <v>1</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E71" s="0" t="n">
         <v>2.86335363152876E-005</v>
@@ -1809,10 +1903,10 @@
         <v>4</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D72" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E72" s="0" t="n">
         <v>0.0148327445015081</v>
@@ -1826,10 +1920,10 @@
         <v>4</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E73" s="0" t="n">
         <v>0.0423018416670973</v>
@@ -1843,10 +1937,10 @@
         <v>2</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="E74" s="0" t="n">
         <v>0.0379316883083251</v>
@@ -1860,10 +1954,10 @@
         <v>3</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E75" s="0" t="n">
         <v>0.0374272936245397</v>
@@ -1877,10 +1971,10 @@
         <v>3</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E76" s="0" t="n">
         <v>0.0108022991106536</v>

</xml_diff>

<commit_message>
zombies_all_anova_passed_cells--used for grant.xlsx updated more.. (manual sorting logged)
</commit_message>
<xml_diff>
--- a/Cortana/cell_list_investigation/zombies_all_anova_passed_cells--used for grant.xlsx
+++ b/Cortana/cell_list_investigation/zombies_all_anova_passed_cells--used for grant.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="103">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -244,6 +244,12 @@
     <t xml:space="preserve">(1650.0, 1800.0)</t>
   </si>
   <si>
+    <t xml:space="preserve">3 or 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">too noisy</t>
+  </si>
+  <si>
     <t xml:space="preserve">(1750.0, 1900.0)</t>
   </si>
   <si>
@@ -266,6 +272,9 @@
   </si>
   <si>
     <t xml:space="preserve">(850.0, 950.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed</t>
   </si>
   <si>
     <t xml:space="preserve">(1500.0, 1600.0)</t>
@@ -1508,6 +1517,12 @@
       <c r="E49" s="0" t="n">
         <v>0.009555414268796</v>
       </c>
+      <c r="F49" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="50" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="n">
@@ -1525,6 +1540,15 @@
       <c r="E50" s="10" t="n">
         <v>0.00580553000234327</v>
       </c>
+      <c r="F50" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="51" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="n">
@@ -1542,6 +1566,15 @@
       <c r="E51" s="10" t="n">
         <v>0.001540377255957</v>
       </c>
+      <c r="F51" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="n">
@@ -1559,6 +1592,12 @@
       <c r="E52" s="0" t="n">
         <v>0.01126620279013</v>
       </c>
+      <c r="F52" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="n">
@@ -1568,13 +1607,19 @@
         <v>3</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D53" s="0" t="s">
         <v>64</v>
       </c>
       <c r="E53" s="0" t="n">
         <v>0.0163236212793226</v>
+      </c>
+      <c r="F53" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G53" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1585,13 +1630,19 @@
         <v>3</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D54" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E54" s="0" t="n">
         <v>0.0494787080515314</v>
+      </c>
+      <c r="F54" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="55" s="12" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,7 +1653,7 @@
         <v>4</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D55" s="12" t="s">
         <v>66</v>
@@ -1611,7 +1662,13 @@
         <v>0.00665026125701438</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>77</v>
+        <v>13</v>
+      </c>
+      <c r="G55" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="12" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="56" s="12" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,7 +1688,13 @@
         <v>0.006289624603342</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>77</v>
+        <v>13</v>
+      </c>
+      <c r="G56" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="12" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="57" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1651,7 +1714,13 @@
         <v>0.00763427299537475</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>77</v>
+        <v>13</v>
+      </c>
+      <c r="G57" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="10" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="58" s="10" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1671,7 +1740,13 @@
         <v>0.006514719781525</v>
       </c>
       <c r="F58" s="10" t="s">
-        <v>77</v>
+        <v>13</v>
+      </c>
+      <c r="G58" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="10" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1682,13 +1757,19 @@
         <v>1</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E59" s="0" t="n">
         <v>0.004480491399968</v>
+      </c>
+      <c r="F59" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1699,13 +1780,19 @@
         <v>1</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D60" s="0" t="s">
         <v>12</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>0.011429781534636</v>
+      </c>
+      <c r="F60" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G60" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,6 +1811,12 @@
       <c r="E61" s="0" t="n">
         <v>0.000335148307695</v>
       </c>
+      <c r="F61" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G61" s="0" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="n">
@@ -1733,13 +1826,19 @@
         <v>1</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D62" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>0.0332634341315389</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G62" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1758,6 +1857,9 @@
       <c r="E63" s="0" t="n">
         <v>0.00479018499791497</v>
       </c>
+      <c r="F63" s="0" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="n">
@@ -1767,13 +1869,19 @@
         <v>1</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>0.0156939900887875</v>
+      </c>
+      <c r="F64" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G64" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1787,10 +1895,16 @@
         <v>38</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>0.0307663890018702</v>
+      </c>
+      <c r="F65" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="G65" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1804,7 +1918,7 @@
         <v>11</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>0.0363170926256485</v>
@@ -1818,7 +1932,7 @@
         <v>3</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D67" s="0" t="s">
         <v>64</v>
@@ -1835,10 +1949,10 @@
         <v>4</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E68" s="0" t="n">
         <v>0.0341434537209639</v>
@@ -1852,10 +1966,10 @@
         <v>4</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E69" s="0" t="n">
         <v>0.0420897306933529</v>
@@ -1869,10 +1983,10 @@
         <v>1</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E70" s="0" t="n">
         <v>0.0387635591675108</v>
@@ -1886,10 +2000,10 @@
         <v>1</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E71" s="0" t="n">
         <v>2.86335363152876E-005</v>
@@ -1920,10 +2034,10 @@
         <v>4</v>
       </c>
       <c r="C73" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D73" s="0" t="s">
         <v>94</v>
-      </c>
-      <c r="D73" s="0" t="s">
-        <v>91</v>
       </c>
       <c r="E73" s="0" t="n">
         <v>0.0423018416670973</v>
@@ -1937,10 +2051,10 @@
         <v>2</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E74" s="0" t="n">
         <v>0.0379316883083251</v>
@@ -1954,10 +2068,10 @@
         <v>3</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E75" s="0" t="n">
         <v>0.0374272936245397</v>
@@ -1974,7 +2088,7 @@
         <v>34</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E76" s="0" t="n">
         <v>0.0108022991106536</v>

</xml_diff>